<commit_message>
Daily recap, matchup updates, learning and research 2026-08-30
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-30.xlsx
+++ b/data/k-props/2026-08-30.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="95">
   <si>
     <t>date</t>
   </si>
@@ -145,6 +145,9 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>U</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -154,6 +157,9 @@
     <t>Andrew Alvarez</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
     <t>Tyler Mahle</t>
   </si>
   <si>
@@ -190,6 +196,9 @@
     <t>Parker Messick</t>
   </si>
   <si>
+    <t>W</t>
+  </si>
+  <si>
     <t>Tyler Glasnow</t>
   </si>
   <si>
@@ -208,9 +217,6 @@
     <t>Drew Rasmussen</t>
   </si>
   <si>
-    <t>lineup_unweighted_30d_projected_regulars</t>
-  </si>
-  <si>
     <t>Jordan Hicks</t>
   </si>
   <si>
@@ -223,28 +229,31 @@
     <t>Zebby Matthews</t>
   </si>
   <si>
+    <t>Kumar Rocker</t>
+  </si>
+  <si>
+    <t>Texas Rangers @ Milwaukee Brewers</t>
+  </si>
+  <si>
+    <t>Dustin May</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Braxton Ashcraft</t>
+  </si>
+  <si>
+    <t>Pittsburgh Pirates @ St. Louis Cardinals</t>
+  </si>
+  <si>
     <t>6-7</t>
   </si>
   <si>
-    <t>Kumar Rocker</t>
-  </si>
-  <si>
-    <t>Texas Rangers @ Milwaukee Brewers</t>
-  </si>
-  <si>
-    <t>Dustin May</t>
-  </si>
-  <si>
-    <t>Braxton Ashcraft</t>
-  </si>
-  <si>
-    <t>Pittsburgh Pirates @ St. Louis Cardinals</t>
+    <t>Matthew Liberatore</t>
   </si>
   <si>
     <t>&gt;=7</t>
-  </si>
-  <si>
-    <t>Matthew Liberatore</t>
   </si>
   <si>
     <t>Zac Thornton</t>
@@ -830,22 +839,22 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.1631</v>
+        <v>0.1609</v>
       </c>
       <c r="N2">
         <v>5</v>
       </c>
       <c r="O2">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="P2">
-        <v>4.24</v>
+        <v>4.22</v>
       </c>
       <c r="Q2">
-        <v>0.1122</v>
+        <v>0.0947</v>
       </c>
       <c r="R2">
-        <v>0.329</v>
+        <v>0.322</v>
       </c>
       <c r="S2" t="s">
         <v>43</v>
@@ -860,37 +869,55 @@
         <v>9</v>
       </c>
       <c r="W2">
-        <v>0.206</v>
+        <v>0.2057</v>
       </c>
       <c r="X2">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y2">
         <v>0.9928</v>
       </c>
+      <c r="Z2">
+        <v>2</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>0.66</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
-        <v>3.11</v>
+        <v>2.96</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
-        <v>0.1464</v>
+        <v>0.1396</v>
       </c>
       <c r="AG2">
-        <v>0.9861</v>
+        <v>0.9913</v>
       </c>
       <c r="AH2">
         <v>0.2</v>
       </c>
+      <c r="AI2">
+        <v>-0.96</v>
+      </c>
+      <c r="AJ2">
+        <v>0.96</v>
+      </c>
+      <c r="AK2">
+        <v>-1.16</v>
+      </c>
+      <c r="AL2">
+        <v>1.16</v>
+      </c>
       <c r="AM2">
-        <v>3.31</v>
+        <v>3.16</v>
       </c>
     </row>
     <row r="3" spans="1:39" x14ac:dyDescent="0.25">
@@ -898,7 +925,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>4.5</v>
@@ -919,7 +946,7 @@
         <v>42</v>
       </c>
       <c r="I3">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="J3" t="b">
         <v>0</v>
@@ -931,22 +958,22 @@
         <v>4</v>
       </c>
       <c r="M3">
-        <v>0.2228</v>
+        <v>0.2251</v>
       </c>
       <c r="N3">
         <v>5</v>
       </c>
       <c r="O3">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P3">
-        <v>4.24</v>
+        <v>4.21</v>
       </c>
       <c r="Q3">
-        <v>0.2056</v>
+        <v>0.217</v>
       </c>
       <c r="R3">
-        <v>0.349</v>
+        <v>0.346</v>
       </c>
       <c r="S3" t="s">
         <v>43</v>
@@ -961,37 +988,55 @@
         <v>9</v>
       </c>
       <c r="W3">
-        <v>0.2308</v>
+        <v>0.2305</v>
       </c>
       <c r="X3">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y3">
         <v>0.88</v>
       </c>
+      <c r="Z3">
+        <v>6</v>
+      </c>
       <c r="AA3" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB3">
+        <v>-0.15</v>
       </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD3">
-        <v>3.98</v>
+        <v>4.15</v>
       </c>
       <c r="AE3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF3">
-        <v>0.2168</v>
+        <v>0.2223</v>
       </c>
       <c r="AG3">
-        <v>1.0185</v>
+        <v>1.0238</v>
       </c>
       <c r="AH3">
         <v>0.2</v>
       </c>
+      <c r="AI3">
+        <v>1.85</v>
+      </c>
+      <c r="AJ3">
+        <v>1.85</v>
+      </c>
+      <c r="AK3">
+        <v>1.65</v>
+      </c>
+      <c r="AL3">
+        <v>1.65</v>
+      </c>
       <c r="AM3">
-        <v>4.18</v>
+        <v>4.35</v>
       </c>
     </row>
     <row r="4" spans="1:39" x14ac:dyDescent="0.25">
@@ -999,7 +1044,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4">
         <v>5.5</v>
@@ -1011,7 +1056,7 @@
         <v>110</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G4">
         <v>824876</v>
@@ -1032,22 +1077,22 @@
         <v>5</v>
       </c>
       <c r="M4">
-        <v>0.2254</v>
+        <v>0.2322</v>
       </c>
       <c r="N4">
         <v>5</v>
       </c>
       <c r="O4">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P4">
-        <v>4.2</v>
+        <v>4.17</v>
       </c>
       <c r="Q4">
-        <v>0.2712</v>
+        <v>0.2735</v>
       </c>
       <c r="R4">
-        <v>0.371</v>
+        <v>0.369</v>
       </c>
       <c r="S4" t="s">
         <v>43</v>
@@ -1062,37 +1107,55 @@
         <v>9</v>
       </c>
       <c r="W4">
-        <v>0.2176</v>
+        <v>0.2186</v>
       </c>
       <c r="X4">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y4">
         <v>1.042</v>
       </c>
+      <c r="Z4">
+        <v>9</v>
+      </c>
       <c r="AA4" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB4">
+        <v>0.13</v>
       </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD4">
-        <v>5.28</v>
+        <v>5.43</v>
       </c>
       <c r="AE4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF4">
-        <v>0.2424</v>
+        <v>0.2475</v>
       </c>
       <c r="AG4">
-        <v>0.9255</v>
+        <v>0.9303</v>
       </c>
       <c r="AH4">
         <v>0.2</v>
       </c>
+      <c r="AI4">
+        <v>3.57</v>
+      </c>
+      <c r="AJ4">
+        <v>3.57</v>
+      </c>
+      <c r="AK4">
+        <v>3.37</v>
+      </c>
+      <c r="AL4">
+        <v>3.37</v>
+      </c>
       <c r="AM4">
-        <v>5.48</v>
+        <v>5.63</v>
       </c>
     </row>
     <row r="5" spans="1:39" x14ac:dyDescent="0.25">
@@ -1100,7 +1163,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C5">
         <v>5.5</v>
@@ -1112,7 +1175,7 @@
         <v>-136</v>
       </c>
       <c r="F5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G5">
         <v>823502</v>
@@ -1121,7 +1184,7 @@
         <v>42</v>
       </c>
       <c r="I5">
-        <v>5.1</v>
+        <v>5.2</v>
       </c>
       <c r="J5" t="b">
         <v>0</v>
@@ -1133,22 +1196,22 @@
         <v>5</v>
       </c>
       <c r="M5">
-        <v>0.2383</v>
+        <v>0.2306</v>
       </c>
       <c r="N5">
         <v>5</v>
       </c>
       <c r="O5">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="P5">
-        <v>4.15</v>
+        <v>4.17</v>
       </c>
       <c r="Q5">
-        <v>0.14</v>
+        <v>0.1308</v>
       </c>
       <c r="R5">
-        <v>0.333</v>
+        <v>0.349</v>
       </c>
       <c r="S5" t="s">
         <v>43</v>
@@ -1163,37 +1226,55 @@
         <v>9</v>
       </c>
       <c r="W5">
-        <v>0.2488</v>
+        <v>0.2454</v>
       </c>
       <c r="X5">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y5">
         <v>1.004</v>
       </c>
+      <c r="Z5">
+        <v>2</v>
+      </c>
       <c r="AA5" t="s">
         <v>44</v>
       </c>
+      <c r="AB5">
+        <v>-0.59</v>
+      </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD5">
-        <v>4.88</v>
+        <v>4.71</v>
       </c>
       <c r="AE5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF5">
-        <v>0.2055</v>
+        <v>0.196</v>
       </c>
       <c r="AG5">
-        <v>1.1078</v>
+        <v>1.1136</v>
       </c>
       <c r="AH5">
         <v>0.2</v>
       </c>
+      <c r="AI5">
+        <v>-2.71</v>
+      </c>
+      <c r="AJ5">
+        <v>2.71</v>
+      </c>
+      <c r="AK5">
+        <v>-2.91</v>
+      </c>
+      <c r="AL5">
+        <v>2.91</v>
+      </c>
       <c r="AM5">
-        <v>5.08</v>
+        <v>4.91</v>
       </c>
     </row>
     <row r="6" spans="1:39" x14ac:dyDescent="0.25">
@@ -1201,7 +1282,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C6">
         <v>4.5</v>
@@ -1213,7 +1294,7 @@
         <v>-104</v>
       </c>
       <c r="F6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G6">
         <v>823502</v>
@@ -1234,22 +1315,22 @@
         <v>5</v>
       </c>
       <c r="M6">
-        <v>0.2254</v>
+        <v>0.227</v>
       </c>
       <c r="N6">
         <v>5</v>
       </c>
       <c r="O6">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="P6">
-        <v>4.4</v>
+        <v>4.37</v>
       </c>
       <c r="Q6">
-        <v>0.2202</v>
+        <v>0.2124</v>
       </c>
       <c r="R6">
-        <v>0.353</v>
+        <v>0.361</v>
       </c>
       <c r="S6" t="s">
         <v>43</v>
@@ -1264,37 +1345,55 @@
         <v>7</v>
       </c>
       <c r="W6">
-        <v>0.2139</v>
+        <v>0.2142</v>
       </c>
       <c r="X6">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y6">
         <v>1.0266</v>
       </c>
+      <c r="Z6">
+        <v>7</v>
+      </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB6">
+        <v>0.49</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD6">
-        <v>4.77</v>
+        <v>4.79</v>
       </c>
       <c r="AE6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF6">
-        <v>0.2236</v>
+        <v>0.2217</v>
       </c>
       <c r="AG6">
-        <v>0.9343</v>
+        <v>0.9392</v>
       </c>
       <c r="AH6">
         <v>0.2</v>
       </c>
+      <c r="AI6">
+        <v>2.21</v>
+      </c>
+      <c r="AJ6">
+        <v>2.21</v>
+      </c>
+      <c r="AK6">
+        <v>2.01</v>
+      </c>
+      <c r="AL6">
+        <v>2.01</v>
+      </c>
       <c r="AM6">
-        <v>4.97</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="7" spans="1:39" x14ac:dyDescent="0.25">
@@ -1302,7 +1401,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C7">
         <v>4.5</v>
@@ -1314,7 +1413,7 @@
         <v>128</v>
       </c>
       <c r="F7" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G7">
         <v>822766</v>
@@ -1323,7 +1422,7 @@
         <v>42</v>
       </c>
       <c r="I7">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="J7" t="b">
         <v>0</v>
@@ -1335,22 +1434,22 @@
         <v>4</v>
       </c>
       <c r="M7">
-        <v>0.263</v>
+        <v>0.2602</v>
       </c>
       <c r="N7">
         <v>5</v>
       </c>
       <c r="O7">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="P7">
-        <v>3.97</v>
+        <v>3.98</v>
       </c>
       <c r="Q7">
-        <v>0.2417</v>
+        <v>0.2328</v>
       </c>
       <c r="R7">
-        <v>0.375</v>
+        <v>0.367</v>
       </c>
       <c r="S7" t="s">
         <v>43</v>
@@ -1365,37 +1464,55 @@
         <v>9</v>
       </c>
       <c r="W7">
-        <v>0.1876</v>
+        <v>0.1869</v>
       </c>
       <c r="X7">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y7">
         <v>0.9485</v>
       </c>
+      <c r="Z7">
+        <v>4</v>
+      </c>
       <c r="AA7" t="s">
         <v>44</v>
       </c>
+      <c r="AB7">
+        <v>0.25</v>
+      </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD7">
-        <v>4.62</v>
+        <v>4.55</v>
       </c>
       <c r="AE7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF7">
-        <v>0.255</v>
+        <v>0.2501</v>
       </c>
       <c r="AG7">
-        <v>0.807</v>
+        <v>0.8112</v>
       </c>
       <c r="AH7">
         <v>0.2</v>
       </c>
+      <c r="AI7">
+        <v>-0.55</v>
+      </c>
+      <c r="AJ7">
+        <v>0.55</v>
+      </c>
+      <c r="AK7">
+        <v>-0.75</v>
+      </c>
+      <c r="AL7">
+        <v>0.75</v>
+      </c>
       <c r="AM7">
-        <v>4.82</v>
+        <v>4.75</v>
       </c>
     </row>
     <row r="8" spans="1:39" x14ac:dyDescent="0.25">
@@ -1403,7 +1520,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C8">
         <v>4.5</v>
@@ -1415,16 +1532,16 @@
         <v>-134</v>
       </c>
       <c r="F8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G8">
         <v>822766</v>
       </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I8">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
       <c r="J8" t="b">
         <v>0</v>
@@ -1436,7 +1553,7 @@
         <v>4</v>
       </c>
       <c r="M8">
-        <v>0.16</v>
+        <v>0.1855</v>
       </c>
       <c r="N8">
         <v>5</v>
@@ -1445,10 +1562,10 @@
         <v>108</v>
       </c>
       <c r="P8">
-        <v>4.5</v>
+        <v>4.35</v>
       </c>
       <c r="Q8">
-        <v>0.1667</v>
+        <v>0.213</v>
       </c>
       <c r="R8">
         <v>0.351</v>
@@ -1466,37 +1583,55 @@
         <v>9</v>
       </c>
       <c r="W8">
-        <v>0.2264</v>
+        <v>0.2287</v>
       </c>
       <c r="X8">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y8">
         <v>0.9775</v>
       </c>
+      <c r="Z8">
+        <v>10</v>
+      </c>
       <c r="AA8" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB8">
+        <v>0.1</v>
       </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD8">
-        <v>3.58</v>
+        <v>4.4</v>
       </c>
       <c r="AE8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF8">
-        <v>0.1623</v>
+        <v>0.1951</v>
       </c>
       <c r="AG8">
-        <v>1.2033</v>
+        <v>1.2096</v>
       </c>
       <c r="AH8">
         <v>0.2</v>
       </c>
+      <c r="AI8">
+        <v>5.6</v>
+      </c>
+      <c r="AJ8">
+        <v>5.6</v>
+      </c>
+      <c r="AK8">
+        <v>5.4</v>
+      </c>
+      <c r="AL8">
+        <v>5.4</v>
+      </c>
       <c r="AM8">
-        <v>3.78</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="9" spans="1:39" x14ac:dyDescent="0.25">
@@ -1504,7 +1639,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C9">
         <v>3.5</v>
@@ -1516,7 +1651,7 @@
         <v>116</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G9">
         <v>824393</v>
@@ -1525,7 +1660,7 @@
         <v>42</v>
       </c>
       <c r="I9">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="J9" t="b">
         <v>0</v>
@@ -1537,22 +1672,22 @@
         <v>4</v>
       </c>
       <c r="M9">
-        <v>0.1812</v>
+        <v>0.1782</v>
       </c>
       <c r="N9">
         <v>5</v>
       </c>
       <c r="O9">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="P9">
-        <v>4.26</v>
+        <v>4.3</v>
       </c>
       <c r="Q9">
-        <v>0.1709</v>
+        <v>0.1667</v>
       </c>
       <c r="R9">
-        <v>0.369</v>
+        <v>0.363</v>
       </c>
       <c r="S9" t="s">
         <v>43</v>
@@ -1567,37 +1702,55 @@
         <v>9</v>
       </c>
       <c r="W9">
-        <v>0.2114</v>
+        <v>0.2107</v>
       </c>
       <c r="X9">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y9">
         <v>0.88</v>
       </c>
+      <c r="Z9">
+        <v>2</v>
+      </c>
       <c r="AA9" t="s">
         <v>44</v>
       </c>
+      <c r="AB9">
+        <v>-0.37</v>
+      </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD9">
-        <v>2.98</v>
+        <v>2.93</v>
       </c>
       <c r="AE9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF9">
-        <v>0.1774</v>
+        <v>0.174</v>
       </c>
       <c r="AG9">
-        <v>0.8039</v>
+        <v>0.8081</v>
       </c>
       <c r="AH9">
         <v>0.2</v>
       </c>
+      <c r="AI9">
+        <v>-0.93</v>
+      </c>
+      <c r="AJ9">
+        <v>0.93</v>
+      </c>
+      <c r="AK9">
+        <v>-1.13</v>
+      </c>
+      <c r="AL9">
+        <v>1.13</v>
+      </c>
       <c r="AM9">
-        <v>3.18</v>
+        <v>3.13</v>
       </c>
     </row>
     <row r="10" spans="1:39" x14ac:dyDescent="0.25">
@@ -1605,7 +1758,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C10">
         <v>5.5</v>
@@ -1617,7 +1770,7 @@
         <v>138</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G10">
         <v>824393</v>
@@ -1638,22 +1791,22 @@
         <v>4</v>
       </c>
       <c r="M10">
-        <v>0.2549</v>
+        <v>0.2527</v>
       </c>
       <c r="N10">
         <v>5</v>
       </c>
       <c r="O10">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="P10">
-        <v>3.95</v>
+        <v>3.96</v>
       </c>
       <c r="Q10">
-        <v>0.2931</v>
+        <v>0.2727</v>
       </c>
       <c r="R10">
-        <v>0.367</v>
+        <v>0.377</v>
       </c>
       <c r="S10" t="s">
         <v>43</v>
@@ -1668,37 +1821,55 @@
         <v>9</v>
       </c>
       <c r="W10">
-        <v>0.2135</v>
+        <v>0.2133</v>
       </c>
       <c r="X10">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y10">
         <v>0.9277</v>
       </c>
+      <c r="Z10">
+        <v>5</v>
+      </c>
       <c r="AA10" t="s">
         <v>44</v>
       </c>
+      <c r="AB10">
+        <v>-0.71</v>
+      </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD10">
-        <v>4.7</v>
+        <v>4.59</v>
       </c>
       <c r="AE10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF10">
-        <v>0.2689</v>
+        <v>0.2603</v>
       </c>
       <c r="AG10">
-        <v>0.8011</v>
+        <v>0.8053</v>
       </c>
       <c r="AH10">
         <v>0.2</v>
       </c>
+      <c r="AI10">
+        <v>0.41</v>
+      </c>
+      <c r="AJ10">
+        <v>0.41</v>
+      </c>
+      <c r="AK10">
+        <v>0.21</v>
+      </c>
+      <c r="AL10">
+        <v>0.21</v>
+      </c>
       <c r="AM10">
-        <v>4.9</v>
+        <v>4.79</v>
       </c>
     </row>
     <row r="11" spans="1:39" x14ac:dyDescent="0.25">
@@ -1706,7 +1877,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C11">
         <v>6.5</v>
@@ -1718,7 +1889,7 @@
         <v>-108</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G11">
         <v>824232</v>
@@ -1727,7 +1898,7 @@
         <v>42</v>
       </c>
       <c r="I11">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="J11" t="b">
         <v>0</v>
@@ -1739,22 +1910,22 @@
         <v>5</v>
       </c>
       <c r="M11">
-        <v>0.3314</v>
+        <v>0.3229</v>
       </c>
       <c r="N11">
         <v>5</v>
       </c>
       <c r="O11">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P11">
-        <v>3.78</v>
+        <v>3.72</v>
       </c>
       <c r="Q11">
-        <v>0.3469</v>
+        <v>0.3402</v>
       </c>
       <c r="R11">
-        <v>0.329</v>
+        <v>0.327</v>
       </c>
       <c r="S11" t="s">
         <v>43</v>
@@ -1769,37 +1940,55 @@
         <v>9</v>
       </c>
       <c r="W11">
-        <v>0.2238</v>
+        <v>0.2239</v>
       </c>
       <c r="X11">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y11">
         <v>0.88</v>
       </c>
+      <c r="Z11">
+        <v>6</v>
+      </c>
       <c r="AA11" t="s">
         <v>44</v>
       </c>
+      <c r="AB11">
+        <v>-1.05</v>
+      </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD11">
-        <v>5.3</v>
+        <v>5.25</v>
       </c>
       <c r="AE11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF11">
-        <v>0.3365</v>
+        <v>0.3286</v>
       </c>
       <c r="AG11">
-        <v>0.8469</v>
+        <v>0.8513</v>
       </c>
       <c r="AH11">
         <v>0.2</v>
       </c>
+      <c r="AI11">
+        <v>0.75</v>
+      </c>
+      <c r="AJ11">
+        <v>0.75</v>
+      </c>
+      <c r="AK11">
+        <v>0.55</v>
+      </c>
+      <c r="AL11">
+        <v>0.55</v>
+      </c>
       <c r="AM11">
-        <v>5.5</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="12" spans="1:39" x14ac:dyDescent="0.25">
@@ -1807,7 +1996,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C12">
         <v>4.5</v>
@@ -1819,7 +2008,7 @@
         <v>-137</v>
       </c>
       <c r="F12" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G12">
         <v>824232</v>
@@ -1840,22 +2029,22 @@
         <v>5</v>
       </c>
       <c r="M12">
-        <v>0.1737</v>
+        <v>0.1747</v>
       </c>
       <c r="N12">
         <v>5</v>
       </c>
       <c r="O12">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="P12">
-        <v>4.42</v>
+        <v>4.41</v>
       </c>
       <c r="Q12">
-        <v>0.1397</v>
+        <v>0.1374</v>
       </c>
       <c r="R12">
-        <v>0.405</v>
+        <v>0.396</v>
       </c>
       <c r="S12" t="s">
         <v>43</v>
@@ -1873,34 +2062,52 @@
         <v>0.204</v>
       </c>
       <c r="X12">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y12">
         <v>0.951</v>
       </c>
+      <c r="Z12">
+        <v>5</v>
+      </c>
       <c r="AA12" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB12">
+        <v>-0.59</v>
       </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD12">
-        <v>3.69</v>
+        <v>3.71</v>
       </c>
       <c r="AE12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF12">
         <v>0.1599</v>
       </c>
       <c r="AG12">
-        <v>0.9866</v>
+        <v>0.9917</v>
       </c>
       <c r="AH12">
         <v>0.2</v>
       </c>
+      <c r="AI12">
+        <v>1.29</v>
+      </c>
+      <c r="AJ12">
+        <v>1.29</v>
+      </c>
+      <c r="AK12">
+        <v>1.09</v>
+      </c>
+      <c r="AL12">
+        <v>1.09</v>
+      </c>
       <c r="AM12">
-        <v>3.89</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="13" spans="1:39" x14ac:dyDescent="0.25">
@@ -1908,7 +2115,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C13">
         <v>4.5</v>
@@ -1920,7 +2127,7 @@
         <v>-154</v>
       </c>
       <c r="F13" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G13">
         <v>822933</v>
@@ -1941,7 +2148,7 @@
         <v>3</v>
       </c>
       <c r="M13">
-        <v>0.2033</v>
+        <v>0.2026</v>
       </c>
       <c r="N13">
         <v>5</v>
@@ -1950,10 +2157,10 @@
         <v>110</v>
       </c>
       <c r="P13">
-        <v>4.2</v>
+        <v>4.17</v>
       </c>
       <c r="Q13">
-        <v>0.1909</v>
+        <v>0.1727</v>
       </c>
       <c r="R13">
         <v>0.355</v>
@@ -1971,37 +2178,55 @@
         <v>9</v>
       </c>
       <c r="W13">
-        <v>0.1831</v>
+        <v>0.184</v>
       </c>
       <c r="X13">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y13">
         <v>0.88</v>
       </c>
+      <c r="Z13">
+        <v>4</v>
+      </c>
       <c r="AA13" t="s">
         <v>44</v>
       </c>
+      <c r="AB13">
+        <v>-1.24</v>
+      </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD13">
-        <v>3.16</v>
+        <v>3.06</v>
       </c>
       <c r="AE13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF13">
-        <v>0.1989</v>
+        <v>0.192</v>
       </c>
       <c r="AG13">
-        <v>0.7872</v>
+        <v>0.7913</v>
       </c>
       <c r="AH13">
         <v>0.2</v>
       </c>
+      <c r="AI13">
+        <v>0.94</v>
+      </c>
+      <c r="AJ13">
+        <v>0.94</v>
+      </c>
+      <c r="AK13">
+        <v>0.74</v>
+      </c>
+      <c r="AL13">
+        <v>0.74</v>
+      </c>
       <c r="AM13">
-        <v>3.36</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="14" spans="1:39" x14ac:dyDescent="0.25">
@@ -2009,7 +2234,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C14">
         <v>5.5</v>
@@ -2021,7 +2246,7 @@
         <v>-136</v>
       </c>
       <c r="F14" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G14">
         <v>822933</v>
@@ -2042,67 +2267,85 @@
         <v>3</v>
       </c>
       <c r="M14">
-        <v>0.26</v>
+        <v>0.2596</v>
       </c>
       <c r="N14">
         <v>5</v>
       </c>
       <c r="O14">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="P14">
         <v>3.92</v>
       </c>
       <c r="Q14">
-        <v>0.2793</v>
+        <v>0.2389</v>
       </c>
       <c r="R14">
-        <v>0.357</v>
+        <v>0.361</v>
       </c>
       <c r="S14" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="T14">
-        <v>0.1933</v>
+        <v>0.1892</v>
       </c>
       <c r="U14">
-        <v>0.1962</v>
+        <v>0.1995</v>
       </c>
       <c r="V14">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W14">
-        <v>0.2151</v>
+        <v>0.2161</v>
       </c>
       <c r="X14">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y14">
-        <v>1.0026</v>
+        <v>1.0485</v>
+      </c>
+      <c r="Z14">
+        <v>6</v>
       </c>
       <c r="AA14" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB14">
+        <v>-0.2</v>
       </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD14">
-        <v>5.23</v>
+        <v>5.1</v>
       </c>
       <c r="AE14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF14">
-        <v>0.2669</v>
+        <v>0.2521</v>
       </c>
       <c r="AG14">
-        <v>0.8884</v>
+        <v>0.8737</v>
       </c>
       <c r="AH14">
         <v>0.2</v>
       </c>
+      <c r="AI14">
+        <v>0.9</v>
+      </c>
+      <c r="AJ14">
+        <v>0.9</v>
+      </c>
+      <c r="AK14">
+        <v>0.7</v>
+      </c>
+      <c r="AL14">
+        <v>0.7</v>
+      </c>
       <c r="AM14">
-        <v>5.43</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="15" spans="1:39" x14ac:dyDescent="0.25">
@@ -2110,16 +2353,16 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G15">
         <v>823662</v>
       </c>
       <c r="H15" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I15">
         <v>1</v>
@@ -2134,22 +2377,22 @@
         <v>0</v>
       </c>
       <c r="M15">
-        <v>0.2737</v>
+        <v>0.2717</v>
       </c>
       <c r="N15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O15">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="P15">
-        <v>4.47</v>
+        <v>4.52</v>
       </c>
       <c r="Q15">
-        <v>0.3333</v>
+        <v>0.25</v>
       </c>
       <c r="R15">
-        <v>0.015</v>
+        <v>0.038</v>
       </c>
       <c r="S15" t="s">
         <v>43</v>
@@ -2164,37 +2407,37 @@
         <v>9</v>
       </c>
       <c r="W15">
-        <v>0.2071</v>
+        <v>0.2063</v>
       </c>
       <c r="X15">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y15">
         <v>0.9478</v>
       </c>
       <c r="AA15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD15">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="AE15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF15">
-        <v>0.2746</v>
+        <v>0.2709</v>
       </c>
       <c r="AG15">
-        <v>0.8542</v>
+        <v>0.8587</v>
       </c>
       <c r="AH15">
         <v>0.2</v>
       </c>
       <c r="AM15">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="16" spans="1:39" x14ac:dyDescent="0.25">
@@ -2202,7 +2445,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C16">
         <v>4.5</v>
@@ -2214,7 +2457,7 @@
         <v>112</v>
       </c>
       <c r="F16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G16">
         <v>823662</v>
@@ -2223,7 +2466,7 @@
         <v>42</v>
       </c>
       <c r="I16">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="J16" t="b">
         <v>0</v>
@@ -2235,22 +2478,22 @@
         <v>4</v>
       </c>
       <c r="M16">
-        <v>0.2014</v>
+        <v>0.1991</v>
       </c>
       <c r="N16">
         <v>5</v>
       </c>
       <c r="O16">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="P16">
-        <v>4.22</v>
+        <v>4.17</v>
       </c>
       <c r="Q16">
-        <v>0.2458</v>
+        <v>0.1905</v>
       </c>
       <c r="R16">
-        <v>0.371</v>
+        <v>0.387</v>
       </c>
       <c r="S16" t="s">
         <v>43</v>
@@ -2265,37 +2508,55 @@
         <v>9</v>
       </c>
       <c r="W16">
-        <v>0.2367</v>
+        <v>0.236</v>
       </c>
       <c r="X16">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y16">
         <v>1.098</v>
       </c>
+      <c r="Z16">
+        <v>5</v>
+      </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB16">
+        <v>1.68</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD16">
-        <v>6.54</v>
+        <v>5.98</v>
       </c>
       <c r="AE16" t="s">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="AF16">
-        <v>0.2178</v>
+        <v>0.1958</v>
       </c>
       <c r="AG16">
-        <v>1.1267</v>
+        <v>1.1326</v>
       </c>
       <c r="AH16">
-        <v>-0.35</v>
+        <v>0.2</v>
+      </c>
+      <c r="AI16">
+        <v>-0.98</v>
+      </c>
+      <c r="AJ16">
+        <v>0.98</v>
+      </c>
+      <c r="AK16">
+        <v>-1.18</v>
+      </c>
+      <c r="AL16">
+        <v>1.18</v>
       </c>
       <c r="AM16">
-        <v>6.19</v>
+        <v>6.18</v>
       </c>
     </row>
     <row r="17" spans="1:39" x14ac:dyDescent="0.25">
@@ -2303,7 +2564,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C17">
         <v>4.5</v>
@@ -2315,7 +2576,7 @@
         <v>-102</v>
       </c>
       <c r="F17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G17">
         <v>823740</v>
@@ -2324,7 +2585,7 @@
         <v>42</v>
       </c>
       <c r="I17">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="J17" t="b">
         <v>0</v>
@@ -2336,22 +2597,22 @@
         <v>3</v>
       </c>
       <c r="M17">
-        <v>0.2116</v>
+        <v>0.2175</v>
       </c>
       <c r="N17">
         <v>5</v>
       </c>
       <c r="O17">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="P17">
-        <v>4.37</v>
+        <v>4.4</v>
       </c>
       <c r="Q17">
-        <v>0.2051</v>
+        <v>0.243</v>
       </c>
       <c r="R17">
-        <v>0.369</v>
+        <v>0.349</v>
       </c>
       <c r="S17" t="s">
         <v>43</v>
@@ -2366,37 +2627,55 @@
         <v>9</v>
       </c>
       <c r="W17">
-        <v>0.2145</v>
+        <v>0.2152</v>
       </c>
       <c r="X17">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y17">
         <v>1.0211</v>
       </c>
+      <c r="Z17">
+        <v>7</v>
+      </c>
       <c r="AA17" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB17">
+        <v>1.01</v>
       </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD17">
-        <v>4.93</v>
+        <v>5.31</v>
       </c>
       <c r="AE17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF17">
-        <v>0.2092</v>
+        <v>0.2264</v>
       </c>
       <c r="AG17">
-        <v>1.0666</v>
+        <v>1.0722</v>
       </c>
       <c r="AH17">
         <v>0.2</v>
       </c>
+      <c r="AI17">
+        <v>1.69</v>
+      </c>
+      <c r="AJ17">
+        <v>1.69</v>
+      </c>
+      <c r="AK17">
+        <v>1.49</v>
+      </c>
+      <c r="AL17">
+        <v>1.49</v>
+      </c>
       <c r="AM17">
-        <v>5.13</v>
+        <v>5.51</v>
       </c>
     </row>
     <row r="18" spans="1:39" x14ac:dyDescent="0.25">
@@ -2404,7 +2683,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C18">
         <v>4.5</v>
@@ -2416,7 +2695,7 @@
         <v>113</v>
       </c>
       <c r="F18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G18">
         <v>823740</v>
@@ -2425,7 +2704,7 @@
         <v>42</v>
       </c>
       <c r="I18">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="J18" t="b">
         <v>0</v>
@@ -2437,67 +2716,85 @@
         <v>3</v>
       </c>
       <c r="M18">
-        <v>0.2252</v>
+        <v>0.223</v>
       </c>
       <c r="N18">
         <v>5</v>
       </c>
       <c r="O18">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="P18">
-        <v>4.21</v>
+        <v>4.25</v>
       </c>
       <c r="Q18">
-        <v>0.1807</v>
+        <v>0.1818</v>
       </c>
       <c r="R18">
-        <v>0.293</v>
+        <v>0.306</v>
       </c>
       <c r="S18" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="T18">
-        <v>0.2444</v>
+        <v>0.2289</v>
       </c>
       <c r="U18">
-        <v>0.236</v>
+        <v>0.2321</v>
       </c>
       <c r="V18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W18">
-        <v>0.2229</v>
+        <v>0.2225</v>
       </c>
       <c r="X18">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y18">
-        <v>1.0279</v>
+        <v>1.091</v>
+      </c>
+      <c r="Z18">
+        <v>4</v>
       </c>
       <c r="AA18" t="s">
         <v>44</v>
       </c>
+      <c r="AB18">
+        <v>0.81</v>
+      </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="AD18">
-        <v>5.13</v>
+        <v>5.11</v>
       </c>
       <c r="AE18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF18">
-        <v>0.2121</v>
+        <v>0.2104</v>
       </c>
       <c r="AG18">
-        <v>1.1231</v>
+        <v>1.0573</v>
       </c>
       <c r="AH18">
         <v>0.2</v>
       </c>
+      <c r="AI18">
+        <v>-1.11</v>
+      </c>
+      <c r="AJ18">
+        <v>1.11</v>
+      </c>
+      <c r="AK18">
+        <v>-1.31</v>
+      </c>
+      <c r="AL18">
+        <v>1.31</v>
+      </c>
       <c r="AM18">
-        <v>5.33</v>
+        <v>5.31</v>
       </c>
     </row>
     <row r="19" spans="1:39" x14ac:dyDescent="0.25">
@@ -2505,7 +2802,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C19">
         <v>5.5</v>
@@ -2517,7 +2814,7 @@
         <v>-151</v>
       </c>
       <c r="F19" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G19">
         <v>823010</v>
@@ -2526,7 +2823,7 @@
         <v>42</v>
       </c>
       <c r="I19">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="J19" t="b">
         <v>0</v>
@@ -2538,22 +2835,22 @@
         <v>4</v>
       </c>
       <c r="M19">
-        <v>0.2584</v>
+        <v>0.2543</v>
       </c>
       <c r="N19">
         <v>5</v>
       </c>
       <c r="O19">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="P19">
-        <v>4.01</v>
+        <v>4.02</v>
       </c>
       <c r="Q19">
-        <v>0.2241</v>
+        <v>0.2017</v>
       </c>
       <c r="R19">
-        <v>0.367</v>
+        <v>0.373</v>
       </c>
       <c r="S19" t="s">
         <v>43</v>
@@ -2568,37 +2865,55 @@
         <v>9</v>
       </c>
       <c r="W19">
-        <v>0.2156</v>
+        <v>0.2152</v>
       </c>
       <c r="X19">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y19">
         <v>0.9066</v>
       </c>
+      <c r="Z19">
+        <v>3</v>
+      </c>
       <c r="AA19" t="s">
         <v>44</v>
       </c>
+      <c r="AB19">
+        <v>0.85</v>
+      </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="AD19">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="AE19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AF19">
-        <v>0.2458</v>
+        <v>0.2346</v>
       </c>
       <c r="AG19">
-        <v>1.3109</v>
+        <v>1.3177</v>
       </c>
       <c r="AH19">
-        <v>0</v>
+        <v>-0.35</v>
+      </c>
+      <c r="AI19">
+        <v>-3.7</v>
+      </c>
+      <c r="AJ19">
+        <v>3.7</v>
+      </c>
+      <c r="AK19">
+        <v>-3.35</v>
+      </c>
+      <c r="AL19">
+        <v>3.35</v>
       </c>
       <c r="AM19">
-        <v>7</v>
+        <v>6.35</v>
       </c>
     </row>
     <row r="20" spans="1:39" x14ac:dyDescent="0.25">
@@ -2606,7 +2921,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C20">
         <v>5.5</v>
@@ -2618,7 +2933,7 @@
         <v>102</v>
       </c>
       <c r="F20" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G20">
         <v>823010</v>
@@ -2639,67 +2954,85 @@
         <v>4</v>
       </c>
       <c r="M20">
-        <v>0.2345</v>
+        <v>0.2394</v>
       </c>
       <c r="N20">
         <v>5</v>
       </c>
       <c r="O20">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="P20">
-        <v>4.36</v>
+        <v>4.37</v>
       </c>
       <c r="Q20">
-        <v>0.2991</v>
+        <v>0.3009</v>
       </c>
       <c r="R20">
-        <v>0.349</v>
+        <v>0.361</v>
       </c>
       <c r="S20" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="T20">
-        <v>0.2058</v>
+        <v>0.2947</v>
       </c>
       <c r="U20">
-        <v>0.2431</v>
+        <v>0.2961</v>
       </c>
       <c r="V20">
         <v>9</v>
       </c>
       <c r="W20">
-        <v>0.2623</v>
+        <v>0.2636</v>
       </c>
       <c r="X20">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y20">
-        <v>1.0274</v>
+        <v>1.0901</v>
+      </c>
+      <c r="Z20">
+        <v>9</v>
       </c>
       <c r="AA20" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB20">
+        <v>2.97</v>
       </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD20">
-        <v>5.41</v>
+        <v>8.47</v>
       </c>
       <c r="AE20" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="AF20">
-        <v>0.257</v>
+        <v>0.2616</v>
       </c>
       <c r="AG20">
-        <v>0.9456</v>
+        <v>1.3612</v>
       </c>
       <c r="AH20">
-        <v>0.2</v>
+        <v>0</v>
+      </c>
+      <c r="AI20">
+        <v>0.53</v>
+      </c>
+      <c r="AJ20">
+        <v>0.53</v>
+      </c>
+      <c r="AK20">
+        <v>0.53</v>
+      </c>
+      <c r="AL20">
+        <v>0.53</v>
       </c>
       <c r="AM20">
-        <v>5.61</v>
+        <v>8.47</v>
       </c>
     </row>
     <row r="21" spans="1:39" x14ac:dyDescent="0.25">
@@ -2707,10 +3040,10 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F21" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G21">
         <v>823580</v>
@@ -2731,67 +3064,67 @@
         <v>0</v>
       </c>
       <c r="M21">
-        <v>0.1794</v>
+        <v>0.1837</v>
       </c>
       <c r="N21">
         <v>5</v>
       </c>
       <c r="O21">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="P21">
-        <v>3.96</v>
+        <v>3.99</v>
       </c>
       <c r="Q21">
-        <v>0.1593</v>
+        <v>0.1892</v>
       </c>
       <c r="R21">
-        <v>0.361</v>
+        <v>0.357</v>
       </c>
       <c r="S21" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="T21">
-        <v>0.2095</v>
+        <v>0.1959</v>
       </c>
       <c r="U21">
-        <v>0.2016</v>
+        <v>0.1951</v>
       </c>
       <c r="V21">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W21">
         <v>0.2092</v>
       </c>
       <c r="X21">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y21">
-        <v>0.9839</v>
+        <v>0.9589</v>
       </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD21">
-        <v>3.63</v>
+        <v>3.59</v>
       </c>
       <c r="AE21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF21">
-        <v>0.1721</v>
+        <v>0.1856</v>
       </c>
       <c r="AG21">
-        <v>0.9625</v>
+        <v>0.9047</v>
       </c>
       <c r="AH21">
         <v>0.2</v>
       </c>
       <c r="AM21">
-        <v>3.83</v>
+        <v>3.79</v>
       </c>
     </row>
     <row r="22" spans="1:39" x14ac:dyDescent="0.25">
@@ -2799,7 +3132,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C22">
         <v>4.5</v>
@@ -2811,7 +3144,7 @@
         <v>-113</v>
       </c>
       <c r="F22" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G22">
         <v>824959</v>
@@ -2820,7 +3153,7 @@
         <v>42</v>
       </c>
       <c r="I22">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="J22" t="b">
         <v>0</v>
@@ -2832,67 +3165,85 @@
         <v>3</v>
       </c>
       <c r="M22">
-        <v>0.1522</v>
+        <v>0.1519</v>
       </c>
       <c r="N22">
         <v>5</v>
       </c>
       <c r="O22">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="P22">
-        <v>4.53</v>
+        <v>4.54</v>
       </c>
       <c r="Q22">
-        <v>0.1504</v>
+        <v>0.1624</v>
       </c>
       <c r="R22">
-        <v>0.361</v>
+        <v>0.369</v>
       </c>
       <c r="S22" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="T22">
-        <v>0.2551</v>
+        <v>0.2005</v>
       </c>
       <c r="U22">
-        <v>0.2206</v>
+        <v>0.2011</v>
       </c>
       <c r="V22">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W22">
         <v>0.2138</v>
       </c>
       <c r="X22">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y22">
-        <v>1.0562</v>
+        <v>1.0918</v>
+      </c>
+      <c r="Z22">
+        <v>4</v>
       </c>
       <c r="AA22" t="s">
         <v>44</v>
       </c>
+      <c r="AB22">
+        <v>-0.76</v>
+      </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD22">
-        <v>4.16</v>
+        <v>3.54</v>
       </c>
       <c r="AE22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF22">
-        <v>0.1516</v>
+        <v>0.1558</v>
       </c>
       <c r="AG22">
-        <v>1.1724</v>
+        <v>0.9261</v>
       </c>
       <c r="AH22">
         <v>0.2</v>
       </c>
+      <c r="AI22">
+        <v>0.46</v>
+      </c>
+      <c r="AJ22">
+        <v>0.46</v>
+      </c>
+      <c r="AK22">
+        <v>0.26</v>
+      </c>
+      <c r="AL22">
+        <v>0.26</v>
+      </c>
       <c r="AM22">
-        <v>4.36</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="23" spans="1:39" x14ac:dyDescent="0.25">
@@ -2900,7 +3251,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C23">
         <v>3.5</v>
@@ -2912,7 +3263,7 @@
         <v>128</v>
       </c>
       <c r="F23" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G23">
         <v>824959</v>
@@ -2933,31 +3284,31 @@
         <v>3</v>
       </c>
       <c r="M23">
-        <v>0.1746</v>
+        <v>0.1788</v>
       </c>
       <c r="N23">
         <v>5</v>
       </c>
       <c r="O23">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P23">
-        <v>4.45</v>
+        <v>4.46</v>
       </c>
       <c r="Q23">
-        <v>0.0825</v>
+        <v>0.1224</v>
       </c>
       <c r="R23">
-        <v>0.327</v>
+        <v>0.329</v>
       </c>
       <c r="S23" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="T23">
-        <v>0.2588</v>
+        <v>0.2363</v>
       </c>
       <c r="U23">
-        <v>0.2467</v>
+        <v>0.2538</v>
       </c>
       <c r="V23">
         <v>9</v>
@@ -2966,34 +3317,52 @@
         <v>0.2582</v>
       </c>
       <c r="X23">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y23">
-        <v>1.0149</v>
+        <v>1.0423</v>
+      </c>
+      <c r="Z23">
+        <v>6</v>
       </c>
       <c r="AA23" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB23">
+        <v>0.7</v>
       </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD23">
-        <v>3.93</v>
+        <v>4</v>
       </c>
       <c r="AE23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF23">
-        <v>0.1484</v>
+        <v>0.1603</v>
       </c>
       <c r="AG23">
-        <v>1.1894</v>
+        <v>1.0916</v>
       </c>
       <c r="AH23">
         <v>0.2</v>
       </c>
+      <c r="AI23">
+        <v>2</v>
+      </c>
+      <c r="AJ23">
+        <v>2</v>
+      </c>
+      <c r="AK23">
+        <v>1.8</v>
+      </c>
+      <c r="AL23">
+        <v>1.8</v>
+      </c>
       <c r="AM23">
-        <v>4.13</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="24" spans="1:39" x14ac:dyDescent="0.25">
@@ -3001,7 +3370,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C24">
         <v>7.5</v>
@@ -3013,7 +3382,7 @@
         <v>-152</v>
       </c>
       <c r="F24" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="G24">
         <v>823987</v>
@@ -3034,31 +3403,31 @@
         <v>4</v>
       </c>
       <c r="M24">
-        <v>0.2966</v>
+        <v>0.2939</v>
       </c>
       <c r="N24">
         <v>5</v>
       </c>
       <c r="O24">
-        <v>103</v>
+        <v>121</v>
       </c>
       <c r="P24">
-        <v>4.01</v>
+        <v>4.02</v>
       </c>
       <c r="Q24">
-        <v>0.2427</v>
+        <v>0.2314</v>
       </c>
       <c r="R24">
-        <v>0.34</v>
+        <v>0.377</v>
       </c>
       <c r="S24" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="T24">
-        <v>0.275</v>
+        <v>0.278</v>
       </c>
       <c r="U24">
-        <v>0.2515</v>
+        <v>0.2778</v>
       </c>
       <c r="V24">
         <v>9</v>
@@ -3067,34 +3436,52 @@
         <v>0.2519</v>
       </c>
       <c r="X24">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y24">
-        <v>1.032</v>
+        <v>1.0363</v>
+      </c>
+      <c r="Z24">
+        <v>6</v>
       </c>
       <c r="AA24" t="s">
         <v>44</v>
       </c>
+      <c r="AB24">
+        <v>0.7</v>
+      </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="AD24">
-        <v>8.23</v>
+        <v>8.2</v>
       </c>
       <c r="AE24" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AF24">
-        <v>0.2783</v>
+        <v>0.2703</v>
       </c>
       <c r="AG24">
-        <v>1.2637</v>
+        <v>1.2842</v>
       </c>
       <c r="AH24">
         <v>0</v>
       </c>
+      <c r="AI24">
+        <v>-2.2</v>
+      </c>
+      <c r="AJ24">
+        <v>2.2</v>
+      </c>
+      <c r="AK24">
+        <v>-2.2</v>
+      </c>
+      <c r="AL24">
+        <v>2.2</v>
+      </c>
       <c r="AM24">
-        <v>8.23</v>
+        <v>8.2</v>
       </c>
     </row>
     <row r="25" spans="1:39" x14ac:dyDescent="0.25">
@@ -3102,7 +3489,7 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C25">
         <v>5.5</v>
@@ -3114,7 +3501,7 @@
         <v>-118</v>
       </c>
       <c r="F25" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="G25">
         <v>823987</v>
@@ -3123,7 +3510,7 @@
         <v>42</v>
       </c>
       <c r="I25">
-        <v>4.5</v>
+        <v>4.8</v>
       </c>
       <c r="J25" t="b">
         <v>0</v>
@@ -3135,31 +3522,31 @@
         <v>4</v>
       </c>
       <c r="M25">
-        <v>0.2242</v>
+        <v>0.224</v>
       </c>
       <c r="N25">
         <v>5</v>
       </c>
       <c r="O25">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="P25">
-        <v>4.58</v>
+        <v>4.47</v>
       </c>
       <c r="Q25">
-        <v>0.2211</v>
+        <v>0.233</v>
       </c>
       <c r="R25">
-        <v>0.322</v>
+        <v>0.34</v>
       </c>
       <c r="S25" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="T25">
-        <v>0.1497</v>
+        <v>0.1811</v>
       </c>
       <c r="U25">
-        <v>0.1531</v>
+        <v>0.1806</v>
       </c>
       <c r="V25">
         <v>9</v>
@@ -3168,34 +3555,52 @@
         <v>0.2241</v>
       </c>
       <c r="X25">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y25">
-        <v>0.9624</v>
+        <v>1.0213</v>
+      </c>
+      <c r="Z25">
+        <v>6</v>
       </c>
       <c r="AA25" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB25">
+        <v>-1.16</v>
       </c>
       <c r="AC25" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="AD25">
-        <v>3.05</v>
+        <v>4.14</v>
       </c>
       <c r="AE25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF25">
-        <v>0.2232</v>
+        <v>0.227</v>
       </c>
       <c r="AG25">
-        <v>0.6878</v>
+        <v>0.8363</v>
       </c>
       <c r="AH25">
         <v>0.2</v>
       </c>
+      <c r="AI25">
+        <v>1.86</v>
+      </c>
+      <c r="AJ25">
+        <v>1.86</v>
+      </c>
+      <c r="AK25">
+        <v>1.66</v>
+      </c>
+      <c r="AL25">
+        <v>1.66</v>
+      </c>
       <c r="AM25">
-        <v>3.25</v>
+        <v>4.34</v>
       </c>
     </row>
     <row r="26" spans="1:39" x14ac:dyDescent="0.25">
@@ -3203,7 +3608,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C26">
         <v>6.5</v>
@@ -3215,7 +3620,7 @@
         <v>-161</v>
       </c>
       <c r="F26" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="G26">
         <v>824636</v>
@@ -3254,13 +3659,13 @@
         <v>0.359</v>
       </c>
       <c r="S26" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="T26">
-        <v>0.2093</v>
+        <v>0.2298</v>
       </c>
       <c r="U26">
-        <v>0.2026</v>
+        <v>0.2106</v>
       </c>
       <c r="V26">
         <v>9</v>
@@ -3269,34 +3674,52 @@
         <v>0.215</v>
       </c>
       <c r="X26">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y26">
-        <v>0.9711</v>
+        <v>0.9315</v>
+      </c>
+      <c r="Z26">
+        <v>7</v>
       </c>
       <c r="AA26" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB26">
+        <v>-0.11</v>
       </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD26">
-        <v>6.37</v>
+        <v>6.74</v>
       </c>
       <c r="AE26" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="AF26">
         <v>0.3008</v>
       </c>
       <c r="AG26">
-        <v>0.9616</v>
+        <v>1.0613</v>
       </c>
       <c r="AH26">
         <v>-0.35</v>
       </c>
+      <c r="AI26">
+        <v>0.26</v>
+      </c>
+      <c r="AJ26">
+        <v>0.26</v>
+      </c>
+      <c r="AK26">
+        <v>0.61</v>
+      </c>
+      <c r="AL26">
+        <v>0.61</v>
+      </c>
       <c r="AM26">
-        <v>6.02</v>
+        <v>6.39</v>
       </c>
     </row>
     <row r="27" spans="1:39" x14ac:dyDescent="0.25">
@@ -3304,7 +3727,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C27">
         <v>5.5</v>
@@ -3316,7 +3739,7 @@
         <v>124</v>
       </c>
       <c r="F27" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="G27">
         <v>824636</v>
@@ -3355,49 +3778,67 @@
         <v>0.344</v>
       </c>
       <c r="S27" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="T27">
-        <v>0.2637</v>
+        <v>0.2303</v>
       </c>
       <c r="U27">
-        <v>0.2645</v>
+        <v>0.2603</v>
       </c>
       <c r="V27">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W27">
         <v>0.2479</v>
       </c>
       <c r="X27">
-        <v>0.2176</v>
+        <v>0.2165</v>
       </c>
       <c r="Y27">
-        <v>1.0681</v>
+        <v>1.12</v>
+      </c>
+      <c r="Z27">
+        <v>4</v>
       </c>
       <c r="AA27" t="s">
         <v>44</v>
       </c>
+      <c r="AB27">
+        <v>1.58</v>
+      </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="AD27">
-        <v>7.7</v>
+        <v>7.08</v>
       </c>
       <c r="AE27" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AF27">
         <v>0.2611</v>
       </c>
       <c r="AG27">
-        <v>1.2117</v>
+        <v>1.0637</v>
       </c>
       <c r="AH27">
         <v>0</v>
       </c>
+      <c r="AI27">
+        <v>-3.08</v>
+      </c>
+      <c r="AJ27">
+        <v>3.08</v>
+      </c>
+      <c r="AK27">
+        <v>-3.08</v>
+      </c>
+      <c r="AL27">
+        <v>3.08</v>
+      </c>
       <c r="AM27">
-        <v>7.7</v>
+        <v>7.08</v>
       </c>
     </row>
     <row r="28" spans="1:39" x14ac:dyDescent="0.25">
@@ -3405,7 +3846,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C28">
         <v>3.5</v>
@@ -3417,31 +3858,31 @@
         <v>103</v>
       </c>
       <c r="F28" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L28">
         <v>5</v>
       </c>
       <c r="S28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:39" x14ac:dyDescent="0.25">
@@ -3449,7 +3890,7 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C29">
         <v>3.5</v>
@@ -3461,31 +3902,31 @@
         <v>-109</v>
       </c>
       <c r="F29" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L29">
         <v>3</v>
       </c>
       <c r="S29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:39" x14ac:dyDescent="0.25">
@@ -3493,7 +3934,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C30">
         <v>3.5</v>
@@ -3505,31 +3946,31 @@
         <v>103</v>
       </c>
       <c r="F30" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L30">
         <v>3</v>
       </c>
       <c r="S30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>